<commit_message>
first sound fx, improved char collision, image button start
</commit_message>
<xml_diff>
--- a/char creating.xlsx
+++ b/char creating.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utufi-my.sharepoint.com/personal/nisine_utu_fi/Documents/Koulu/Tietotekniikka/Harjoitustyö/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="65" documentId="11_F25DC773A252ABDACC10483FA95C7D745BDE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0869DB38-0BCD-4C24-8257-E08B2CB2A4E9}"/>
+  <xr:revisionPtr revIDLastSave="109" documentId="11_F25DC773A252ABDACC10483FA95C7D745BDE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43AD2FFF-B4AD-4F4C-9F30-3778835A3F54}"/>
   <bookViews>
-    <workbookView xWindow="19500" yWindow="990" windowWidth="12870" windowHeight="18795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12825" yWindow="4665" windowWidth="9855" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
   <si>
     <t>GAME</t>
   </si>
@@ -97,6 +97,45 @@
   </si>
   <si>
     <t>mult</t>
+  </si>
+  <si>
+    <t>cap for tackling players</t>
+  </si>
+  <si>
+    <t>right</t>
+  </si>
+  <si>
+    <t>left</t>
+  </si>
+  <si>
+    <t>angles</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>max</t>
+  </si>
+  <si>
+    <t>grace</t>
+  </si>
+  <si>
+    <t>min_angle</t>
+  </si>
+  <si>
+    <t>max_angle</t>
+  </si>
+  <si>
+    <t>bumped angle</t>
+  </si>
+  <si>
+    <t>VALUE</t>
+  </si>
+  <si>
+    <t>CAP</t>
+  </si>
+  <si>
+    <t>Angle change</t>
   </si>
 </sst>
 </file>
@@ -120,10 +159,19 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -132,9 +180,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -150,6 +199,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -415,10 +468,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:H20"/>
+  <dimension ref="B2:H40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.140625" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
@@ -531,7 +587,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
         <v>9</v>
       </c>
@@ -539,7 +595,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" t="str">
         <f>B4</f>
         <v>bg_char_creating</v>
@@ -553,7 +609,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>4</v>
       </c>
@@ -566,7 +622,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>11</v>
       </c>
@@ -578,6 +634,146 @@
         <f>(D19+D7/2-D18)/H4-D8/2</f>
         <v>32</v>
       </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23" t="s">
+        <v>20</v>
+      </c>
+      <c r="F23" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D24">
+        <v>30</v>
+      </c>
+      <c r="E24">
+        <v>40</v>
+      </c>
+      <c r="F24">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>23</v>
+      </c>
+      <c r="F26">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="2"/>
+      <c r="E27" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C28" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E28" t="s">
+        <v>17</v>
+      </c>
+      <c r="F28" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29">
+        <f>D24</f>
+        <v>30</v>
+      </c>
+      <c r="D29" s="2">
+        <v>180</v>
+      </c>
+      <c r="E29">
+        <v>180</v>
+      </c>
+      <c r="F29">
+        <f>360-D24</f>
+        <v>330</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D30" s="2"/>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>22</v>
+      </c>
+      <c r="C31">
+        <f>E24</f>
+        <v>40</v>
+      </c>
+      <c r="D31" s="2">
+        <f>F24</f>
+        <v>75</v>
+      </c>
+      <c r="E31">
+        <f>360-F24</f>
+        <v>285</v>
+      </c>
+      <c r="F31">
+        <f>360-E24</f>
+        <v>320</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D32" s="2"/>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>24</v>
+      </c>
+      <c r="D33" s="2"/>
+      <c r="F33">
+        <f>MAX(MIN(F26,F31),E31)</f>
+        <v>320</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D34" s="2"/>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>25</v>
+      </c>
+      <c r="D35" s="2"/>
+      <c r="F35">
+        <f>F26-F33</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D36" s="2"/>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D37" s="2"/>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D38" s="2"/>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D39" s="2"/>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D40" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>